<commit_message>
feat: add Postman API collection, automation utilities, and manual testing documentation
</commit_message>
<xml_diff>
--- a/manual-testing/manual-test-cases.xlsx
+++ b/manual-testing/manual-test-cases.xlsx
@@ -40,7 +40,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -72,11 +72,6 @@
         <fgColor rgb="007B2C2C"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -96,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -112,9 +107,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3026,52 +3018,52 @@
       </c>
     </row>
     <row r="2" ht="60" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>BUG_001</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>UX_001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Forgot Password</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>'Failed to send OTP' toast on Forgot Password with valid email</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>UX Note: Unclear error message when submitting unregistered email</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>1. Go to /auth/login
 2. Click 'Forgot Password?'
-3. Enter mitesh8767@gmail.com
+3. Enter an unregistered email (e.g., unknown@test.com)
 4. Click Submit</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>OTP sent successfully, confirmation message displayed</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>Toast: 'Failed to send OTP' appears immediately — OTP not delivered</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Should show a clear, user-friendly message (e.g., 'Email not found')</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Displays a generic or vague error message instead of a specific user-friendly prompt</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Low (UX)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>See browser screenshot (DevTools console screenshot)</t>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>